<commit_message>
Checkpoint before assistant change: Update database with surgery data and fix web speedometer.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9DD5E615-1263-4080-94C0-014C218D78DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{251EA1EB-97B9-4F35-9B4B-302E1A6F0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="101">
   <si>
     <t>data</t>
   </si>
@@ -202,94 +202,31 @@
     <t>bloqueio_data</t>
   </si>
   <si>
+    <t>2025-03-10</t>
+  </si>
+  <si>
+    <t>09/03/2025</t>
+  </si>
+  <si>
+    <t>Carlos Eduardo Milani</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Dra. Ana Clara</t>
+  </si>
+  <si>
+    <t>Mariana Moro, Mariana Silva, Assistente Extra, Aline  (extra), Natália  (extra)</t>
+  </si>
+  <si>
+    <t>06:30</t>
+  </si>
+  <si>
     <t>Sim</t>
   </si>
   <si>
     <t>Não</t>
-  </si>
-  <si>
-    <t>2025-03-10</t>
-  </si>
-  <si>
-    <t>09/03/2025</t>
-  </si>
-  <si>
-    <t>Carlos Eduardo Milani</t>
-  </si>
-  <si>
-    <t>Rio de Janeiro</t>
-  </si>
-  <si>
-    <t>Dra. Ana Clara</t>
-  </si>
-  <si>
-    <t>Mariana Moro, Mariana Silva, Assistente Extra, Aline  (extra), Natália  (extra)</t>
-  </si>
-  <si>
-    <t>06:30</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>3414</t>
-  </si>
-  <si>
-    <t>2964</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>450</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>0.85</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>650</t>
-  </si>
-  <si>
-    <t>637</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>1150</t>
-  </si>
-  <si>
-    <t>1027</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>1100</t>
-  </si>
-  <si>
-    <t>49</t>
-  </si>
-  <si>
-    <t>700</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t xml:space="preserve">Nega </t>
@@ -312,6 +249,81 @@
   </si>
   <si>
     <t>{"tipo":"Xilo sem vaso","seringas":"3","comentarios":"A dra aqui faz um bloqueio diferente uma seringa de 3 ml 1,5 de xilo e 1,5 de soro \nE duas seringas  de 1,5 ropi e 1,5 de soro"}</t>
+  </si>
+  <si>
+    <t>2025-03-06</t>
+  </si>
+  <si>
+    <t>05/03/2025</t>
+  </si>
+  <si>
+    <t>Jonas Galatti Carbonera</t>
+  </si>
+  <si>
+    <t>Ribeirão Preto</t>
+  </si>
+  <si>
+    <t>Dr. Daniel</t>
+  </si>
+  <si>
+    <t>Aline, Natália, Ana, thamara (extra)</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>3705</t>
+  </si>
+  <si>
+    <t>0.85</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>750</t>
+  </si>
+  <si>
+    <t>730</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>1250</t>
+  </si>
+  <si>
+    <t>1202</t>
+  </si>
+  <si>
+    <t>1200</t>
+  </si>
+  <si>
+    <t>1186</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>630</t>
+  </si>
+  <si>
+    <t>587</t>
+  </si>
+  <si>
+    <t>thamara</t>
+  </si>
+  <si>
+    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
   </si>
 </sst>
 </file>
@@ -674,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH2"/>
+  <dimension ref="A1:BH3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
@@ -861,148 +873,261 @@
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" t="s">
         <v>62</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>63</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>64</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>65</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>66</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
+        <v>3414</v>
+      </c>
+      <c r="J2">
+        <v>2964</v>
+      </c>
+      <c r="K2">
+        <v>80</v>
+      </c>
+      <c r="L2">
+        <v>450</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>200</v>
+      </c>
+      <c r="O2">
+        <v>200</v>
+      </c>
+      <c r="P2" t="s">
         <v>67</v>
       </c>
-      <c r="G2" t="s">
+      <c r="Q2">
+        <v>0.85</v>
+      </c>
+      <c r="R2">
+        <v>6</v>
+      </c>
+      <c r="S2">
+        <v>3</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>48</v>
+      </c>
+      <c r="V2">
+        <v>650</v>
+      </c>
+      <c r="W2">
+        <v>637</v>
+      </c>
+      <c r="X2">
         <v>68</v>
       </c>
-      <c r="H2" t="s">
+      <c r="Y2">
+        <v>1150</v>
+      </c>
+      <c r="Z2">
+        <v>1027</v>
+      </c>
+      <c r="AA2">
+        <v>64</v>
+      </c>
+      <c r="AB2">
+        <v>1200</v>
+      </c>
+      <c r="AC2">
+        <v>1100</v>
+      </c>
+      <c r="AD2">
+        <v>49</v>
+      </c>
+      <c r="AE2">
+        <v>700</v>
+      </c>
+      <c r="AF2">
+        <v>650</v>
+      </c>
+      <c r="AG2">
+        <v>1</v>
+      </c>
+      <c r="AH2">
+        <v>1</v>
+      </c>
+      <c r="AI2">
+        <v>1</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO2" t="s">
         <v>69</v>
       </c>
-      <c r="I2" t="s">
+      <c r="AP2" t="s">
         <v>70</v>
       </c>
-      <c r="J2" t="s">
+      <c r="AQ2" t="s">
         <v>71</v>
       </c>
-      <c r="K2" t="s">
+      <c r="AR2" t="s">
         <v>72</v>
       </c>
-      <c r="L2" t="s">
+      <c r="AS2" t="s">
         <v>73</v>
       </c>
-      <c r="M2" t="s">
+      <c r="AT2">
+        <v>3</v>
+      </c>
+      <c r="AU2" t="s">
         <v>74</v>
       </c>
-      <c r="N2" t="s">
+      <c r="BH2" t="s">
         <v>75</v>
       </c>
-      <c r="O2" t="s">
-        <v>75</v>
-      </c>
-      <c r="P2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q2" t="s">
+    </row>
+    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>76</v>
       </c>
-      <c r="R2" t="s">
-        <v>69</v>
-      </c>
-      <c r="S2" t="s">
+      <c r="B3" t="s">
         <v>77</v>
       </c>
-      <c r="T2" t="s">
-        <v>74</v>
-      </c>
-      <c r="U2" t="s">
+      <c r="C3" t="s">
         <v>78</v>
       </c>
-      <c r="V2" t="s">
+      <c r="D3" t="s">
         <v>79</v>
       </c>
-      <c r="W2" t="s">
+      <c r="E3" t="s">
         <v>80</v>
       </c>
-      <c r="X2" t="s">
+      <c r="F3" t="s">
         <v>81</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="G3" t="s">
         <v>82</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="H3" t="s">
         <v>83</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="I3" t="s">
         <v>84</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="J3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P3" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q3" t="s">
         <v>85</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="R3" t="s">
         <v>86</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="T3" t="s">
         <v>87</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="U3" t="s">
         <v>88</v>
       </c>
-      <c r="AF2" t="s">
-        <v>79</v>
-      </c>
-      <c r="AG2" t="s">
+      <c r="V3" t="s">
         <v>89</v>
       </c>
-      <c r="AH2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>61</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AO2" t="s">
+      <c r="W3" t="s">
         <v>90</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="X3" t="s">
         <v>91</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="Y3" t="s">
         <v>92</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="Z3" t="s">
         <v>93</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AA3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AB3" t="s">
         <v>94</v>
       </c>
-      <c r="AT2" t="s">
-        <v>77</v>
-      </c>
-      <c r="AU2" t="s">
+      <c r="AC3" t="s">
         <v>95</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="AD3" t="s">
         <v>96</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migrate to a Flask SQLAlchemy database; fix data loss on update.
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e858dfef-e9b8-4fe5-a2eb-b434090118f2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/bf8c4c22-abdf-40af-9137-fa8cd4cf9554.jpg
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{251EA1EB-97B9-4F35-9B4B-302E1A6F0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{84F8D3F4-4D14-4251-8588-271262C0CA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="109">
   <si>
     <t>data</t>
   </si>
@@ -272,58 +272,82 @@
     <t>08:00</t>
   </si>
   <si>
+    <t>thamara</t>
+  </si>
+  <si>
+    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+  </si>
+  <si>
+    <t>adnan jamil el homoui</t>
+  </si>
+  <si>
+    <t>Dr. Arthur</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
-    <t>3705</t>
+    <t>2850</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>310</t>
+  </si>
+  <si>
+    <t>240</t>
   </si>
   <si>
     <t>0.85</t>
   </si>
   <si>
-    <t>8</t>
+    <t>3</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>630</t>
+  </si>
+  <si>
+    <t>585</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>1120</t>
+  </si>
+  <si>
+    <t>1090</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>1200</t>
+  </si>
+  <si>
+    <t>1060</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>750</t>
+  </si>
+  <si>
+    <t>885</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>750</t>
-  </si>
-  <si>
-    <t>730</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>1250</t>
-  </si>
-  <si>
-    <t>1202</t>
-  </si>
-  <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>1186</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>630</t>
-  </si>
-  <si>
-    <t>587</t>
-  </si>
-  <si>
-    <t>thamara</t>
-  </si>
-  <si>
-    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+    <t>hipertenso em uso de alodipina</t>
   </si>
 </sst>
 </file>
@@ -686,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH3"/>
+  <dimension ref="A1:BH4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
@@ -1039,95 +1063,217 @@
       <c r="G3" t="s">
         <v>82</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>3705</v>
+      </c>
+      <c r="J3">
+        <v>3705</v>
+      </c>
+      <c r="P3" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q3">
+        <v>0.85</v>
+      </c>
+      <c r="R3">
+        <v>8</v>
+      </c>
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3">
+        <v>55</v>
+      </c>
+      <c r="V3">
+        <v>750</v>
+      </c>
+      <c r="W3">
+        <v>730</v>
+      </c>
+      <c r="X3">
+        <v>76</v>
+      </c>
+      <c r="Y3">
+        <v>1250</v>
+      </c>
+      <c r="Z3">
+        <v>1202</v>
+      </c>
+      <c r="AA3">
+        <v>76</v>
+      </c>
+      <c r="AB3">
+        <v>1200</v>
+      </c>
+      <c r="AC3">
+        <v>1186</v>
+      </c>
+      <c r="AD3">
+        <v>48</v>
+      </c>
+      <c r="AE3">
+        <v>630</v>
+      </c>
+      <c r="AF3">
+        <v>587</v>
+      </c>
+      <c r="AG3">
+        <v>1</v>
+      </c>
+      <c r="AH3">
+        <v>1</v>
+      </c>
+      <c r="AI3">
+        <v>1</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ3" t="s">
         <v>83</v>
       </c>
-      <c r="I3" t="s">
+      <c r="AS3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH3" t="s">
         <v>84</v>
       </c>
-      <c r="J3" t="s">
+    </row>
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" t="s">
+        <v>88</v>
+      </c>
+      <c r="J4" t="s">
+        <v>89</v>
+      </c>
+      <c r="N4" t="s">
+        <v>90</v>
+      </c>
+      <c r="O4" t="s">
+        <v>91</v>
+      </c>
+      <c r="P4" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>92</v>
+      </c>
+      <c r="R4" t="s">
+        <v>93</v>
+      </c>
+      <c r="T4" t="s">
+        <v>94</v>
+      </c>
+      <c r="U4" t="s">
+        <v>95</v>
+      </c>
+      <c r="V4" t="s">
+        <v>96</v>
+      </c>
+      <c r="W4" t="s">
+        <v>97</v>
+      </c>
+      <c r="X4" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>100</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>104</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>105</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>106</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>107</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>107</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>93</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>108</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH4" t="s">
         <v>84</v>
-      </c>
-      <c r="P3" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R3" t="s">
-        <v>86</v>
-      </c>
-      <c r="T3" t="s">
-        <v>87</v>
-      </c>
-      <c r="U3" t="s">
-        <v>88</v>
-      </c>
-      <c r="V3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X3" t="s">
-        <v>91</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>92</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>99</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Excel data import functionality.  Adds an endpoint to ingest data from an Excel file into the PostgreSQL database.
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e858dfef-e9b8-4fe5-a2eb-b434090118f2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8c7417ff-25e3-4894-9a88-ca4d88413804/d4b6553d-3ac2-4ce9-b65b-2be70e4ae9d8.jpg
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84F8D3F4-4D14-4251-8588-271262C0CA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A647D91A-C13F-4CC8-B549-50007849D54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="130">
   <si>
     <t>data</t>
   </si>
@@ -284,70 +284,136 @@
     <t>Dr. Arthur</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2850</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>310</t>
-  </si>
-  <si>
-    <t>240</t>
-  </si>
-  <si>
-    <t>0.85</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>630</t>
-  </si>
-  <si>
-    <t>585</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>1120</t>
-  </si>
-  <si>
-    <t>1090</t>
+    <t>hipertenso em uso de alodipina</t>
+  </si>
+  <si>
+    <t>has</t>
+  </si>
+  <si>
+    <t>Hygor Henrique Bonfante</t>
+  </si>
+  <si>
+    <t>nega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+</t>
+  </si>
+  <si>
+    <t>2025-03-13</t>
+  </si>
+  <si>
+    <t>12/03/2025</t>
+  </si>
+  <si>
+    <t>Eduardo Roncaglia de Carvalho</t>
+  </si>
+  <si>
+    <t>Aline, Natália, thamara (extra)</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
+</t>
+  </si>
+  <si>
+    <t>Weslei Diego Pavini</t>
+  </si>
+  <si>
+    <t>Ana, angelica  (extra), larissa (extra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angelica </t>
+  </si>
+  <si>
+    <t>larissa</t>
+  </si>
+  <si>
+    <t>2025-03-07</t>
+  </si>
+  <si>
+    <t>06/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+  </si>
+  <si>
+    <t>2025-03-11</t>
+  </si>
+  <si>
+    <t>10/03/2025</t>
+  </si>
+  <si>
+    <t>José Antônio Tonetto Neto</t>
+  </si>
+  <si>
+    <t>6.5</t>
+  </si>
+  <si>
+    <t>3498</t>
+  </si>
+  <si>
+    <t>808</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>1190</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>64</t>
   </si>
   <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>668</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>1050</t>
+  </si>
+  <si>
+    <t>930</t>
+  </si>
+  <si>
+    <t>1300</t>
+  </si>
+  <si>
     <t>1200</t>
   </si>
   <si>
-    <t>1060</t>
-  </si>
-  <si>
-    <t>53</t>
+    <t>57</t>
   </si>
   <si>
     <t>750</t>
   </si>
   <si>
-    <t>885</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>hipertenso em uso de alodipina</t>
+    <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
   </si>
 </sst>
 </file>
@@ -710,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH4"/>
+  <dimension ref="A1:BH10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
@@ -1176,95 +1242,95 @@
       <c r="G4" t="s">
         <v>82</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>2850</v>
+      </c>
+      <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="N4">
+        <v>310</v>
+      </c>
+      <c r="O4">
+        <v>240</v>
+      </c>
+      <c r="P4" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q4">
+        <v>0.85</v>
+      </c>
+      <c r="R4">
+        <v>3</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>45</v>
+      </c>
+      <c r="V4">
+        <v>630</v>
+      </c>
+      <c r="W4">
+        <v>585</v>
+      </c>
+      <c r="X4">
+        <v>60</v>
+      </c>
+      <c r="Y4">
+        <v>1120</v>
+      </c>
+      <c r="Z4">
+        <v>1090</v>
+      </c>
+      <c r="AA4">
+        <v>64</v>
+      </c>
+      <c r="AB4">
+        <v>1200</v>
+      </c>
+      <c r="AC4">
+        <v>1060</v>
+      </c>
+      <c r="AD4">
+        <v>53</v>
+      </c>
+      <c r="AE4">
+        <v>750</v>
+      </c>
+      <c r="AF4">
+        <v>885</v>
+      </c>
+      <c r="AG4">
+        <v>1</v>
+      </c>
+      <c r="AH4">
+        <v>1</v>
+      </c>
+      <c r="AI4">
+        <v>3</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO4" t="s">
         <v>87</v>
-      </c>
-      <c r="I4" t="s">
-        <v>88</v>
-      </c>
-      <c r="J4" t="s">
-        <v>89</v>
-      </c>
-      <c r="N4" t="s">
-        <v>90</v>
-      </c>
-      <c r="O4" t="s">
-        <v>91</v>
-      </c>
-      <c r="P4" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>92</v>
-      </c>
-      <c r="R4" t="s">
-        <v>93</v>
-      </c>
-      <c r="T4" t="s">
-        <v>94</v>
-      </c>
-      <c r="U4" t="s">
-        <v>95</v>
-      </c>
-      <c r="V4" t="s">
-        <v>96</v>
-      </c>
-      <c r="W4" t="s">
-        <v>97</v>
-      </c>
-      <c r="X4" t="s">
-        <v>98</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>99</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>100</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>101</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>102</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>103</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>104</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>105</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>93</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>108</v>
       </c>
       <c r="AQ4" t="s">
         <v>83</v>
@@ -1273,6 +1339,777 @@
         <v>68</v>
       </c>
       <c r="BH4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>3400</v>
+      </c>
+      <c r="J5">
+        <v>2850</v>
+      </c>
+      <c r="K5">
+        <v>100</v>
+      </c>
+      <c r="N5">
+        <v>310</v>
+      </c>
+      <c r="O5">
+        <v>239</v>
+      </c>
+      <c r="P5" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q5">
+        <v>0.85</v>
+      </c>
+      <c r="R5">
+        <v>3</v>
+      </c>
+      <c r="T5">
+        <v>-2</v>
+      </c>
+      <c r="U5">
+        <v>45</v>
+      </c>
+      <c r="V5">
+        <v>630</v>
+      </c>
+      <c r="W5">
+        <v>585</v>
+      </c>
+      <c r="X5">
+        <v>60</v>
+      </c>
+      <c r="Y5">
+        <v>1120</v>
+      </c>
+      <c r="Z5">
+        <v>1090</v>
+      </c>
+      <c r="AA5">
+        <v>64</v>
+      </c>
+      <c r="AB5">
+        <v>1200</v>
+      </c>
+      <c r="AC5">
+        <v>1060</v>
+      </c>
+      <c r="AD5">
+        <v>53</v>
+      </c>
+      <c r="AE5">
+        <v>750</v>
+      </c>
+      <c r="AF5">
+        <v>665</v>
+      </c>
+      <c r="AG5">
+        <v>1</v>
+      </c>
+      <c r="AH5">
+        <v>1</v>
+      </c>
+      <c r="AI5">
+        <v>3</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>3572</v>
+      </c>
+      <c r="J6">
+        <v>3162</v>
+      </c>
+      <c r="K6">
+        <v>106</v>
+      </c>
+      <c r="N6">
+        <v>210</v>
+      </c>
+      <c r="O6">
+        <v>2</v>
+      </c>
+      <c r="P6" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q6">
+        <v>0.85</v>
+      </c>
+      <c r="R6">
+        <v>5</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <v>45</v>
+      </c>
+      <c r="V6">
+        <v>400</v>
+      </c>
+      <c r="W6">
+        <v>370</v>
+      </c>
+      <c r="X6">
+        <v>72</v>
+      </c>
+      <c r="Y6">
+        <v>1450</v>
+      </c>
+      <c r="Z6">
+        <v>1365</v>
+      </c>
+      <c r="AA6">
+        <v>76</v>
+      </c>
+      <c r="AB6">
+        <v>1200</v>
+      </c>
+      <c r="AC6">
+        <v>1170</v>
+      </c>
+      <c r="AD6">
+        <v>48</v>
+      </c>
+      <c r="AE6">
+        <v>700</v>
+      </c>
+      <c r="AF6">
+        <v>667</v>
+      </c>
+      <c r="AG6">
+        <v>1</v>
+      </c>
+      <c r="AH6">
+        <v>2</v>
+      </c>
+      <c r="AI6">
+        <v>2</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>91</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>3655</v>
+      </c>
+      <c r="J7">
+        <v>2610</v>
+      </c>
+      <c r="K7">
+        <v>105</v>
+      </c>
+      <c r="L7">
+        <v>840</v>
+      </c>
+      <c r="M7">
+        <v>200</v>
+      </c>
+      <c r="P7" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q7">
+        <v>0.85</v>
+      </c>
+      <c r="R7">
+        <v>4</v>
+      </c>
+      <c r="S7">
+        <v>5</v>
+      </c>
+      <c r="T7">
+        <v>1</v>
+      </c>
+      <c r="U7">
+        <v>49</v>
+      </c>
+      <c r="V7">
+        <v>630</v>
+      </c>
+      <c r="W7">
+        <v>585</v>
+      </c>
+      <c r="X7">
+        <v>81</v>
+      </c>
+      <c r="Y7">
+        <v>1300</v>
+      </c>
+      <c r="Z7">
+        <v>1249</v>
+      </c>
+      <c r="AA7">
+        <v>72</v>
+      </c>
+      <c r="AB7">
+        <v>1300</v>
+      </c>
+      <c r="AC7">
+        <v>1217</v>
+      </c>
+      <c r="AD7">
+        <v>48</v>
+      </c>
+      <c r="AE7">
+        <v>670</v>
+      </c>
+      <c r="AF7">
+        <v>604</v>
+      </c>
+      <c r="AG7">
+        <v>1</v>
+      </c>
+      <c r="AH7">
+        <v>2</v>
+      </c>
+      <c r="AI7">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>99</v>
+      </c>
+      <c r="G8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>3800</v>
+      </c>
+      <c r="J8">
+        <v>3560</v>
+      </c>
+      <c r="K8">
+        <v>76</v>
+      </c>
+      <c r="L8">
+        <v>240</v>
+      </c>
+      <c r="N8">
+        <v>100</v>
+      </c>
+      <c r="O8">
+        <v>98</v>
+      </c>
+      <c r="P8" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q8">
+        <v>0.85</v>
+      </c>
+      <c r="R8">
+        <v>7</v>
+      </c>
+      <c r="S8">
+        <v>2</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="U8">
+        <v>62</v>
+      </c>
+      <c r="V8">
+        <v>630</v>
+      </c>
+      <c r="W8">
+        <v>600</v>
+      </c>
+      <c r="X8">
+        <v>93</v>
+      </c>
+      <c r="Y8">
+        <v>1350</v>
+      </c>
+      <c r="Z8">
+        <v>1300</v>
+      </c>
+      <c r="AA8">
+        <v>88</v>
+      </c>
+      <c r="AB8">
+        <v>1708</v>
+      </c>
+      <c r="AC8">
+        <v>1508</v>
+      </c>
+      <c r="AD8">
+        <v>54</v>
+      </c>
+      <c r="AE8">
+        <v>400</v>
+      </c>
+      <c r="AF8">
+        <v>320</v>
+      </c>
+      <c r="AG8">
+        <v>2</v>
+      </c>
+      <c r="AH8">
+        <v>2</v>
+      </c>
+      <c r="AI8">
+        <v>2</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9">
+        <v>6.5</v>
+      </c>
+      <c r="I9">
+        <v>3737</v>
+      </c>
+      <c r="J9">
+        <v>3737</v>
+      </c>
+      <c r="K9">
+        <v>80</v>
+      </c>
+      <c r="P9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q9">
+        <v>0.85</v>
+      </c>
+      <c r="R9">
+        <v>7</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9">
+        <v>62</v>
+      </c>
+      <c r="V9">
+        <v>630</v>
+      </c>
+      <c r="W9">
+        <v>600</v>
+      </c>
+      <c r="X9">
+        <v>72</v>
+      </c>
+      <c r="Y9">
+        <v>1470</v>
+      </c>
+      <c r="Z9">
+        <v>1400</v>
+      </c>
+      <c r="AA9">
+        <v>68</v>
+      </c>
+      <c r="AB9">
+        <v>1470</v>
+      </c>
+      <c r="AC9">
+        <v>1400</v>
+      </c>
+      <c r="AD9">
+        <v>49</v>
+      </c>
+      <c r="AE9">
+        <v>420</v>
+      </c>
+      <c r="AF9">
+        <v>387</v>
+      </c>
+      <c r="AG9">
+        <v>2</v>
+      </c>
+      <c r="AH9">
+        <v>3</v>
+      </c>
+      <c r="AI9">
+        <v>2</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>105</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I10" t="s">
+        <v>110</v>
+      </c>
+      <c r="J10" t="s">
+        <v>111</v>
+      </c>
+      <c r="K10" t="s">
+        <v>112</v>
+      </c>
+      <c r="L10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M10" t="s">
+        <v>114</v>
+      </c>
+      <c r="P10" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R10" t="s">
+        <v>116</v>
+      </c>
+      <c r="S10" t="s">
+        <v>117</v>
+      </c>
+      <c r="T10" t="s">
+        <v>118</v>
+      </c>
+      <c r="U10" t="s">
+        <v>119</v>
+      </c>
+      <c r="V10" t="s">
+        <v>120</v>
+      </c>
+      <c r="W10" t="s">
+        <v>121</v>
+      </c>
+      <c r="X10" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>122</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>125</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>126</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>120</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>129</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH10" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update surgical report data.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{251EA1EB-97B9-4F35-9B4B-302E1A6F0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A647D91A-C13F-4CC8-B549-50007849D54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="130">
   <si>
     <t>data</t>
   </si>
@@ -272,58 +272,148 @@
     <t>08:00</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>3705</t>
-  </si>
-  <si>
-    <t>0.85</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>thamara</t>
+  </si>
+  <si>
+    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+  </si>
+  <si>
+    <t>adnan jamil el homoui</t>
+  </si>
+  <si>
+    <t>Dr. Arthur</t>
+  </si>
+  <si>
+    <t>hipertenso em uso de alodipina</t>
+  </si>
+  <si>
+    <t>has</t>
+  </si>
+  <si>
+    <t>Hygor Henrique Bonfante</t>
+  </si>
+  <si>
+    <t>nega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 2 e 3. Fios de médio comprimento e médio 
+</t>
+  </si>
+  <si>
+    <t>2025-03-13</t>
+  </si>
+  <si>
+    <t>12/03/2025</t>
+  </si>
+  <si>
+    <t>Eduardo Roncaglia de Carvalho</t>
+  </si>
+  <si>
+    <t>Aline, Natália, thamara (extra)</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 2  e 3 . Fios grossos  e médio . 
+</t>
+  </si>
+  <si>
+    <t>Weslei Diego Pavini</t>
+  </si>
+  <si>
+    <t>Ana, angelica  (extra), larissa (extra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angelica </t>
+  </si>
+  <si>
+    <t>larissa</t>
+  </si>
+  <si>
+    <t>2025-03-07</t>
+  </si>
+  <si>
+    <t>06/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maurício Ronaldo Ribeiro </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fio 1 e 2 Fios fino e longo.</t>
+  </si>
+  <si>
+    <t>2025-03-11</t>
+  </si>
+  <si>
+    <t>10/03/2025</t>
+  </si>
+  <si>
+    <t>José Antônio Tonetto Neto</t>
+  </si>
+  <si>
+    <t>6.5</t>
+  </si>
+  <si>
+    <t>3498</t>
+  </si>
+  <si>
+    <t>808</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>1190</t>
+  </si>
+  <si>
+    <t>0.95</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>55</t>
+    <t>64</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>668</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>1050</t>
+  </si>
+  <si>
+    <t>930</t>
+  </si>
+  <si>
+    <t>1300</t>
+  </si>
+  <si>
+    <t>1200</t>
+  </si>
+  <si>
+    <t>57</t>
   </si>
   <si>
     <t>750</t>
   </si>
   <si>
-    <t>730</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>1250</t>
-  </si>
-  <si>
-    <t>1202</t>
-  </si>
-  <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>1186</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>630</t>
-  </si>
-  <si>
-    <t>587</t>
-  </si>
-  <si>
-    <t>thamara</t>
-  </si>
-  <si>
-    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+    <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
   </si>
 </sst>
 </file>
@@ -686,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH3"/>
+  <dimension ref="A1:BH10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
@@ -1039,95 +1129,988 @@
       <c r="G3" t="s">
         <v>82</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>3705</v>
+      </c>
+      <c r="J3">
+        <v>3705</v>
+      </c>
+      <c r="P3" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q3">
+        <v>0.85</v>
+      </c>
+      <c r="R3">
+        <v>8</v>
+      </c>
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3">
+        <v>55</v>
+      </c>
+      <c r="V3">
+        <v>750</v>
+      </c>
+      <c r="W3">
+        <v>730</v>
+      </c>
+      <c r="X3">
+        <v>76</v>
+      </c>
+      <c r="Y3">
+        <v>1250</v>
+      </c>
+      <c r="Z3">
+        <v>1202</v>
+      </c>
+      <c r="AA3">
+        <v>76</v>
+      </c>
+      <c r="AB3">
+        <v>1200</v>
+      </c>
+      <c r="AC3">
+        <v>1186</v>
+      </c>
+      <c r="AD3">
+        <v>48</v>
+      </c>
+      <c r="AE3">
+        <v>630</v>
+      </c>
+      <c r="AF3">
+        <v>587</v>
+      </c>
+      <c r="AG3">
+        <v>1</v>
+      </c>
+      <c r="AH3">
+        <v>1</v>
+      </c>
+      <c r="AI3">
+        <v>1</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ3" t="s">
         <v>83</v>
       </c>
-      <c r="I3" t="s">
+      <c r="AS3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH3" t="s">
         <v>84</v>
       </c>
-      <c r="J3" t="s">
+    </row>
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H4">
+        <v>5</v>
+      </c>
+      <c r="I4">
+        <v>2850</v>
+      </c>
+      <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="N4">
+        <v>310</v>
+      </c>
+      <c r="O4">
+        <v>240</v>
+      </c>
+      <c r="P4" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q4">
+        <v>0.85</v>
+      </c>
+      <c r="R4">
+        <v>3</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>45</v>
+      </c>
+      <c r="V4">
+        <v>630</v>
+      </c>
+      <c r="W4">
+        <v>585</v>
+      </c>
+      <c r="X4">
+        <v>60</v>
+      </c>
+      <c r="Y4">
+        <v>1120</v>
+      </c>
+      <c r="Z4">
+        <v>1090</v>
+      </c>
+      <c r="AA4">
+        <v>64</v>
+      </c>
+      <c r="AB4">
+        <v>1200</v>
+      </c>
+      <c r="AC4">
+        <v>1060</v>
+      </c>
+      <c r="AD4">
+        <v>53</v>
+      </c>
+      <c r="AE4">
+        <v>750</v>
+      </c>
+      <c r="AF4">
+        <v>885</v>
+      </c>
+      <c r="AG4">
+        <v>1</v>
+      </c>
+      <c r="AH4">
+        <v>1</v>
+      </c>
+      <c r="AI4">
+        <v>3</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>87</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH4" t="s">
         <v>84</v>
       </c>
-      <c r="P3" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q3" t="s">
+    </row>
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
         <v>85</v>
       </c>
-      <c r="R3" t="s">
+      <c r="D5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" t="s">
         <v>86</v>
       </c>
-      <c r="T3" t="s">
-        <v>87</v>
-      </c>
-      <c r="U3" t="s">
+      <c r="F5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>3400</v>
+      </c>
+      <c r="J5">
+        <v>2850</v>
+      </c>
+      <c r="K5">
+        <v>100</v>
+      </c>
+      <c r="N5">
+        <v>310</v>
+      </c>
+      <c r="O5">
+        <v>239</v>
+      </c>
+      <c r="P5" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q5">
+        <v>0.85</v>
+      </c>
+      <c r="R5">
+        <v>3</v>
+      </c>
+      <c r="T5">
+        <v>-2</v>
+      </c>
+      <c r="U5">
+        <v>45</v>
+      </c>
+      <c r="V5">
+        <v>630</v>
+      </c>
+      <c r="W5">
+        <v>585</v>
+      </c>
+      <c r="X5">
+        <v>60</v>
+      </c>
+      <c r="Y5">
+        <v>1120</v>
+      </c>
+      <c r="Z5">
+        <v>1090</v>
+      </c>
+      <c r="AA5">
+        <v>64</v>
+      </c>
+      <c r="AB5">
+        <v>1200</v>
+      </c>
+      <c r="AC5">
+        <v>1060</v>
+      </c>
+      <c r="AD5">
+        <v>53</v>
+      </c>
+      <c r="AE5">
+        <v>750</v>
+      </c>
+      <c r="AF5">
+        <v>665</v>
+      </c>
+      <c r="AG5">
+        <v>1</v>
+      </c>
+      <c r="AH5">
+        <v>1</v>
+      </c>
+      <c r="AI5">
+        <v>3</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO5" t="s">
         <v>88</v>
       </c>
-      <c r="V3" t="s">
+      <c r="AQ5" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
         <v>89</v>
       </c>
-      <c r="W3" t="s">
+      <c r="D6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>3572</v>
+      </c>
+      <c r="J6">
+        <v>3162</v>
+      </c>
+      <c r="K6">
+        <v>106</v>
+      </c>
+      <c r="N6">
+        <v>210</v>
+      </c>
+      <c r="O6">
+        <v>2</v>
+      </c>
+      <c r="P6" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q6">
+        <v>0.85</v>
+      </c>
+      <c r="R6">
+        <v>5</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="U6">
+        <v>45</v>
+      </c>
+      <c r="V6">
+        <v>400</v>
+      </c>
+      <c r="W6">
+        <v>370</v>
+      </c>
+      <c r="X6">
+        <v>72</v>
+      </c>
+      <c r="Y6">
+        <v>1450</v>
+      </c>
+      <c r="Z6">
+        <v>1365</v>
+      </c>
+      <c r="AA6">
+        <v>76</v>
+      </c>
+      <c r="AB6">
+        <v>1200</v>
+      </c>
+      <c r="AC6">
+        <v>1170</v>
+      </c>
+      <c r="AD6">
+        <v>48</v>
+      </c>
+      <c r="AE6">
+        <v>700</v>
+      </c>
+      <c r="AF6">
+        <v>667</v>
+      </c>
+      <c r="AG6">
+        <v>1</v>
+      </c>
+      <c r="AH6">
+        <v>2</v>
+      </c>
+      <c r="AI6">
+        <v>2</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO6" t="s">
         <v>90</v>
       </c>
-      <c r="X3" t="s">
+      <c r="AP6" t="s">
         <v>91</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="AQ6" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>92</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="B7" t="s">
         <v>93</v>
       </c>
-      <c r="AA3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AB3" t="s">
+      <c r="C7" t="s">
         <v>94</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="D7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" t="s">
         <v>95</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="G7" t="s">
         <v>96</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7">
+        <v>3655</v>
+      </c>
+      <c r="J7">
+        <v>2610</v>
+      </c>
+      <c r="K7">
+        <v>105</v>
+      </c>
+      <c r="L7">
+        <v>840</v>
+      </c>
+      <c r="M7">
+        <v>200</v>
+      </c>
+      <c r="P7" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q7">
+        <v>0.85</v>
+      </c>
+      <c r="R7">
+        <v>4</v>
+      </c>
+      <c r="S7">
+        <v>5</v>
+      </c>
+      <c r="T7">
+        <v>1</v>
+      </c>
+      <c r="U7">
+        <v>49</v>
+      </c>
+      <c r="V7">
+        <v>630</v>
+      </c>
+      <c r="W7">
+        <v>585</v>
+      </c>
+      <c r="X7">
+        <v>81</v>
+      </c>
+      <c r="Y7">
+        <v>1300</v>
+      </c>
+      <c r="Z7">
+        <v>1249</v>
+      </c>
+      <c r="AA7">
+        <v>72</v>
+      </c>
+      <c r="AB7">
+        <v>1300</v>
+      </c>
+      <c r="AC7">
+        <v>1217</v>
+      </c>
+      <c r="AD7">
+        <v>48</v>
+      </c>
+      <c r="AE7">
+        <v>670</v>
+      </c>
+      <c r="AF7">
+        <v>604</v>
+      </c>
+      <c r="AG7">
+        <v>1</v>
+      </c>
+      <c r="AH7">
+        <v>2</v>
+      </c>
+      <c r="AI7">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP7" t="s">
         <v>97</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AQ7" t="s">
+        <v>83</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
         <v>98</v>
       </c>
-      <c r="AG3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>87</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AQ3" t="s">
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
         <v>99</v>
       </c>
-      <c r="AS3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BH3" t="s">
+      <c r="G8" t="s">
+        <v>82</v>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8">
+        <v>3800</v>
+      </c>
+      <c r="J8">
+        <v>3560</v>
+      </c>
+      <c r="K8">
+        <v>76</v>
+      </c>
+      <c r="L8">
+        <v>240</v>
+      </c>
+      <c r="N8">
         <v>100</v>
+      </c>
+      <c r="O8">
+        <v>98</v>
+      </c>
+      <c r="P8" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q8">
+        <v>0.85</v>
+      </c>
+      <c r="R8">
+        <v>7</v>
+      </c>
+      <c r="S8">
+        <v>2</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="U8">
+        <v>62</v>
+      </c>
+      <c r="V8">
+        <v>630</v>
+      </c>
+      <c r="W8">
+        <v>600</v>
+      </c>
+      <c r="X8">
+        <v>93</v>
+      </c>
+      <c r="Y8">
+        <v>1350</v>
+      </c>
+      <c r="Z8">
+        <v>1300</v>
+      </c>
+      <c r="AA8">
+        <v>88</v>
+      </c>
+      <c r="AB8">
+        <v>1708</v>
+      </c>
+      <c r="AC8">
+        <v>1508</v>
+      </c>
+      <c r="AD8">
+        <v>54</v>
+      </c>
+      <c r="AE8">
+        <v>400</v>
+      </c>
+      <c r="AF8">
+        <v>320</v>
+      </c>
+      <c r="AG8">
+        <v>2</v>
+      </c>
+      <c r="AH8">
+        <v>2</v>
+      </c>
+      <c r="AI8">
+        <v>2</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9">
+        <v>6.5</v>
+      </c>
+      <c r="I9">
+        <v>3737</v>
+      </c>
+      <c r="J9">
+        <v>3737</v>
+      </c>
+      <c r="K9">
+        <v>80</v>
+      </c>
+      <c r="P9" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q9">
+        <v>0.85</v>
+      </c>
+      <c r="R9">
+        <v>7</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9">
+        <v>62</v>
+      </c>
+      <c r="V9">
+        <v>630</v>
+      </c>
+      <c r="W9">
+        <v>600</v>
+      </c>
+      <c r="X9">
+        <v>72</v>
+      </c>
+      <c r="Y9">
+        <v>1470</v>
+      </c>
+      <c r="Z9">
+        <v>1400</v>
+      </c>
+      <c r="AA9">
+        <v>68</v>
+      </c>
+      <c r="AB9">
+        <v>1470</v>
+      </c>
+      <c r="AC9">
+        <v>1400</v>
+      </c>
+      <c r="AD9">
+        <v>49</v>
+      </c>
+      <c r="AE9">
+        <v>420</v>
+      </c>
+      <c r="AF9">
+        <v>387</v>
+      </c>
+      <c r="AG9">
+        <v>2</v>
+      </c>
+      <c r="AH9">
+        <v>3</v>
+      </c>
+      <c r="AI9">
+        <v>2</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>105</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G10" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I10" t="s">
+        <v>110</v>
+      </c>
+      <c r="J10" t="s">
+        <v>111</v>
+      </c>
+      <c r="K10" t="s">
+        <v>112</v>
+      </c>
+      <c r="L10" t="s">
+        <v>113</v>
+      </c>
+      <c r="M10" t="s">
+        <v>114</v>
+      </c>
+      <c r="P10" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R10" t="s">
+        <v>116</v>
+      </c>
+      <c r="S10" t="s">
+        <v>117</v>
+      </c>
+      <c r="T10" t="s">
+        <v>118</v>
+      </c>
+      <c r="U10" t="s">
+        <v>119</v>
+      </c>
+      <c r="V10" t="s">
+        <v>120</v>
+      </c>
+      <c r="W10" t="s">
+        <v>121</v>
+      </c>
+      <c r="X10" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>122</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>125</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>126</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>120</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>116</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>129</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>100</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH10" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Add patient data and backup files.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A647D91A-C13F-4CC8-B549-50007849D54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902E6E4D-B17F-4CB6-9A55-B0B5418C474E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="129">
   <si>
     <t>data</t>
   </si>
@@ -285,9 +285,6 @@
   </si>
   <si>
     <t>hipertenso em uso de alodipina</t>
-  </si>
-  <si>
-    <t>has</t>
   </si>
   <si>
     <t>Hygor Henrique Bonfante</t>
@@ -776,8 +773,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH10"/>
+  <dimension ref="A1:BH9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1350,7 +1352,7 @@
         <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D5" t="s">
         <v>79</v>
@@ -1368,19 +1370,19 @@
         <v>5</v>
       </c>
       <c r="I5">
-        <v>3400</v>
+        <v>3572</v>
       </c>
       <c r="J5">
-        <v>2850</v>
+        <v>3162</v>
       </c>
       <c r="K5">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="N5">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="O5">
-        <v>239</v>
+        <v>2</v>
       </c>
       <c r="P5" t="s">
         <v>68</v>
@@ -1389,61 +1391,61 @@
         <v>0.85</v>
       </c>
       <c r="R5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T5">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="U5">
         <v>45</v>
       </c>
       <c r="V5">
-        <v>630</v>
+        <v>400</v>
       </c>
       <c r="W5">
-        <v>585</v>
+        <v>370</v>
       </c>
       <c r="X5">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="Y5">
-        <v>1120</v>
+        <v>1450</v>
       </c>
       <c r="Z5">
-        <v>1090</v>
+        <v>1365</v>
       </c>
       <c r="AA5">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="AB5">
         <v>1200</v>
       </c>
       <c r="AC5">
-        <v>1060</v>
+        <v>1170</v>
       </c>
       <c r="AD5">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AE5">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="AF5">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="AG5">
         <v>1</v>
       </c>
       <c r="AH5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ5" t="s">
         <v>68</v>
       </c>
       <c r="AK5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AL5" t="s">
         <v>68</v>
@@ -1455,7 +1457,10 @@
         <v>68</v>
       </c>
       <c r="AO5" t="s">
-        <v>88</v>
+        <v>89</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>90</v>
       </c>
       <c r="AQ5" t="s">
         <v>83</v>
@@ -1469,43 +1474,43 @@
     </row>
     <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
         <v>79</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="G6" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H6">
         <v>5</v>
       </c>
       <c r="I6">
-        <v>3572</v>
+        <v>3655</v>
       </c>
       <c r="J6">
-        <v>3162</v>
+        <v>2610</v>
       </c>
       <c r="K6">
-        <v>106</v>
-      </c>
-      <c r="N6">
-        <v>210</v>
-      </c>
-      <c r="O6">
-        <v>2</v>
+        <v>105</v>
+      </c>
+      <c r="L6">
+        <v>840</v>
+      </c>
+      <c r="M6">
+        <v>200</v>
       </c>
       <c r="P6" t="s">
         <v>68</v>
@@ -1514,46 +1519,49 @@
         <v>0.85</v>
       </c>
       <c r="R6">
+        <v>4</v>
+      </c>
+      <c r="S6">
         <v>5</v>
       </c>
       <c r="T6">
         <v>1</v>
       </c>
       <c r="U6">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="V6">
-        <v>400</v>
+        <v>630</v>
       </c>
       <c r="W6">
-        <v>370</v>
+        <v>585</v>
       </c>
       <c r="X6">
+        <v>81</v>
+      </c>
+      <c r="Y6">
+        <v>1300</v>
+      </c>
+      <c r="Z6">
+        <v>1249</v>
+      </c>
+      <c r="AA6">
         <v>72</v>
       </c>
-      <c r="Y6">
-        <v>1450</v>
-      </c>
-      <c r="Z6">
-        <v>1365</v>
-      </c>
-      <c r="AA6">
-        <v>76</v>
-      </c>
       <c r="AB6">
-        <v>1200</v>
+        <v>1300</v>
       </c>
       <c r="AC6">
-        <v>1170</v>
+        <v>1217</v>
       </c>
       <c r="AD6">
         <v>48</v>
       </c>
       <c r="AE6">
-        <v>700</v>
+        <v>670</v>
       </c>
       <c r="AF6">
-        <v>667</v>
+        <v>604</v>
       </c>
       <c r="AG6">
         <v>1</v>
@@ -1562,7 +1570,7 @@
         <v>2</v>
       </c>
       <c r="AI6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ6" t="s">
         <v>68</v>
@@ -1580,10 +1588,10 @@
         <v>68</v>
       </c>
       <c r="AO6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AP6" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="AQ6" t="s">
         <v>83</v>
@@ -1597,43 +1605,46 @@
     </row>
     <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>79</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G7" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="H7">
         <v>5</v>
       </c>
       <c r="I7">
-        <v>3655</v>
+        <v>3800</v>
       </c>
       <c r="J7">
-        <v>2610</v>
+        <v>3560</v>
       </c>
       <c r="K7">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="L7">
-        <v>840</v>
-      </c>
-      <c r="M7">
-        <v>200</v>
+        <v>240</v>
+      </c>
+      <c r="N7">
+        <v>100</v>
+      </c>
+      <c r="O7">
+        <v>98</v>
       </c>
       <c r="P7" t="s">
         <v>68</v>
@@ -1642,58 +1653,58 @@
         <v>0.85</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T7">
         <v>1</v>
       </c>
       <c r="U7">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="V7">
         <v>630</v>
       </c>
       <c r="W7">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="X7">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="Y7">
+        <v>1350</v>
+      </c>
+      <c r="Z7">
         <v>1300</v>
       </c>
-      <c r="Z7">
-        <v>1249</v>
-      </c>
       <c r="AA7">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="AB7">
-        <v>1300</v>
+        <v>1708</v>
       </c>
       <c r="AC7">
-        <v>1217</v>
+        <v>1508</v>
       </c>
       <c r="AD7">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="AE7">
-        <v>670</v>
+        <v>400</v>
       </c>
       <c r="AF7">
-        <v>604</v>
+        <v>320</v>
       </c>
       <c r="AG7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH7">
         <v>2</v>
       </c>
       <c r="AI7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ7" t="s">
         <v>68</v>
@@ -1710,14 +1721,11 @@
       <c r="AN7" t="s">
         <v>68</v>
       </c>
-      <c r="AO7" t="s">
-        <v>90</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>97</v>
-      </c>
       <c r="AQ7" t="s">
-        <v>83</v>
+        <v>99</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>100</v>
       </c>
       <c r="AS7" t="s">
         <v>68</v>
@@ -1728,13 +1736,13 @@
     </row>
     <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
         <v>79</v>
@@ -1743,31 +1751,22 @@
         <v>86</v>
       </c>
       <c r="F8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G8" t="s">
         <v>82</v>
       </c>
       <c r="H8">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="I8">
-        <v>3800</v>
+        <v>3737</v>
       </c>
       <c r="J8">
-        <v>3560</v>
+        <v>3737</v>
       </c>
       <c r="K8">
-        <v>76</v>
-      </c>
-      <c r="L8">
-        <v>240</v>
-      </c>
-      <c r="N8">
-        <v>100</v>
-      </c>
-      <c r="O8">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="P8" t="s">
         <v>68</v>
@@ -1778,9 +1777,6 @@
       <c r="R8">
         <v>7</v>
       </c>
-      <c r="S8">
-        <v>2</v>
-      </c>
       <c r="T8">
         <v>1</v>
       </c>
@@ -1794,37 +1790,37 @@
         <v>600</v>
       </c>
       <c r="X8">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="Y8">
-        <v>1350</v>
+        <v>1470</v>
       </c>
       <c r="Z8">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="AA8">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="AB8">
-        <v>1708</v>
+        <v>1470</v>
       </c>
       <c r="AC8">
-        <v>1508</v>
+        <v>1400</v>
       </c>
       <c r="AD8">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="AE8">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="AF8">
-        <v>320</v>
+        <v>387</v>
       </c>
       <c r="AG8">
         <v>2</v>
       </c>
       <c r="AH8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI8">
         <v>2</v>
@@ -1844,11 +1840,14 @@
       <c r="AN8" t="s">
         <v>68</v>
       </c>
+      <c r="AP8" t="s">
+        <v>104</v>
+      </c>
       <c r="AQ8" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR8" t="s">
         <v>100</v>
-      </c>
-      <c r="AR8" t="s">
-        <v>101</v>
       </c>
       <c r="AS8" t="s">
         <v>68</v>
@@ -1859,97 +1858,106 @@
     </row>
     <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
         <v>79</v>
       </c>
       <c r="E9" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G9" t="s">
         <v>82</v>
       </c>
-      <c r="H9">
-        <v>6.5</v>
-      </c>
-      <c r="I9">
-        <v>3737</v>
-      </c>
-      <c r="J9">
-        <v>3737</v>
-      </c>
-      <c r="K9">
-        <v>80</v>
+      <c r="H9" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" t="s">
+        <v>109</v>
+      </c>
+      <c r="J9" t="s">
+        <v>110</v>
+      </c>
+      <c r="K9" t="s">
+        <v>111</v>
+      </c>
+      <c r="L9" t="s">
+        <v>112</v>
+      </c>
+      <c r="M9" t="s">
+        <v>113</v>
       </c>
       <c r="P9" t="s">
         <v>68</v>
       </c>
-      <c r="Q9">
-        <v>0.85</v>
-      </c>
-      <c r="R9">
-        <v>7</v>
-      </c>
-      <c r="T9">
-        <v>1</v>
-      </c>
-      <c r="U9">
-        <v>62</v>
-      </c>
-      <c r="V9">
-        <v>630</v>
-      </c>
-      <c r="W9">
-        <v>600</v>
-      </c>
-      <c r="X9">
-        <v>72</v>
-      </c>
-      <c r="Y9">
-        <v>1470</v>
-      </c>
-      <c r="Z9">
-        <v>1400</v>
-      </c>
-      <c r="AA9">
-        <v>68</v>
-      </c>
-      <c r="AB9">
-        <v>1470</v>
-      </c>
-      <c r="AC9">
-        <v>1400</v>
-      </c>
-      <c r="AD9">
-        <v>49</v>
-      </c>
-      <c r="AE9">
-        <v>420</v>
-      </c>
-      <c r="AF9">
-        <v>387</v>
-      </c>
-      <c r="AG9">
-        <v>2</v>
-      </c>
-      <c r="AH9">
-        <v>3</v>
-      </c>
-      <c r="AI9">
-        <v>2</v>
+      <c r="Q9" t="s">
+        <v>114</v>
+      </c>
+      <c r="R9" t="s">
+        <v>115</v>
+      </c>
+      <c r="S9" t="s">
+        <v>116</v>
+      </c>
+      <c r="T9" t="s">
+        <v>117</v>
+      </c>
+      <c r="U9" t="s">
+        <v>118</v>
+      </c>
+      <c r="V9" t="s">
+        <v>119</v>
+      </c>
+      <c r="W9" t="s">
+        <v>120</v>
+      </c>
+      <c r="X9" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>122</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>124</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>125</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>126</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>127</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>119</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>117</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>115</v>
       </c>
       <c r="AJ9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AK9" t="s">
         <v>68</v>
@@ -1963,153 +1971,22 @@
       <c r="AN9" t="s">
         <v>68</v>
       </c>
+      <c r="AO9" t="s">
+        <v>89</v>
+      </c>
       <c r="AP9" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="AQ9" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR9" t="s">
         <v>100</v>
       </c>
-      <c r="AR9" t="s">
-        <v>101</v>
-      </c>
       <c r="AS9" t="s">
         <v>68</v>
       </c>
       <c r="BH9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>106</v>
-      </c>
-      <c r="B10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" t="s">
-        <v>108</v>
-      </c>
-      <c r="D10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" t="s">
-        <v>80</v>
-      </c>
-      <c r="F10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G10" t="s">
-        <v>82</v>
-      </c>
-      <c r="H10" t="s">
-        <v>109</v>
-      </c>
-      <c r="I10" t="s">
-        <v>110</v>
-      </c>
-      <c r="J10" t="s">
-        <v>111</v>
-      </c>
-      <c r="K10" t="s">
-        <v>112</v>
-      </c>
-      <c r="L10" t="s">
-        <v>113</v>
-      </c>
-      <c r="M10" t="s">
-        <v>114</v>
-      </c>
-      <c r="P10" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>115</v>
-      </c>
-      <c r="R10" t="s">
-        <v>116</v>
-      </c>
-      <c r="S10" t="s">
-        <v>117</v>
-      </c>
-      <c r="T10" t="s">
-        <v>118</v>
-      </c>
-      <c r="U10" t="s">
-        <v>119</v>
-      </c>
-      <c r="V10" t="s">
-        <v>120</v>
-      </c>
-      <c r="W10" t="s">
-        <v>121</v>
-      </c>
-      <c r="X10" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>124</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>122</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>125</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>126</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>127</v>
-      </c>
-      <c r="AE10" t="s">
-        <v>128</v>
-      </c>
-      <c r="AF10" t="s">
-        <v>120</v>
-      </c>
-      <c r="AG10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AJ10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>90</v>
-      </c>
-      <c r="AP10" t="s">
-        <v>129</v>
-      </c>
-      <c r="AQ10" t="s">
-        <v>100</v>
-      </c>
-      <c r="AR10" t="s">
-        <v>101</v>
-      </c>
-      <c r="AS10" t="s">
-        <v>68</v>
-      </c>
-      <c r="BH10" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update surgical report with additional patient data (8 to 13 patients).
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902E6E4D-B17F-4CB6-9A55-B0B5418C474E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{846924BB-0F6A-4F6A-B5F5-401829AAEA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="131">
   <si>
     <t>data</t>
   </si>
@@ -202,89 +202,49 @@
     <t>bloqueio_data</t>
   </si>
   <si>
-    <t>2025-03-10</t>
-  </si>
-  <si>
-    <t>09/03/2025</t>
-  </si>
-  <si>
-    <t>Carlos Eduardo Milani</t>
-  </si>
-  <si>
-    <t>Rio de Janeiro</t>
-  </si>
-  <si>
-    <t>Dra. Ana Clara</t>
-  </si>
-  <si>
-    <t>Mariana Moro, Mariana Silva, Assistente Extra, Aline  (extra), Natália  (extra)</t>
-  </si>
-  <si>
-    <t>06:30</t>
+    <t>2025-03-06</t>
+  </si>
+  <si>
+    <t>05/03/2025</t>
+  </si>
+  <si>
+    <t>Jonas Galatti Carbonera</t>
+  </si>
+  <si>
+    <t>Ribeirão Preto</t>
+  </si>
+  <si>
+    <t>Dr. Daniel</t>
+  </si>
+  <si>
+    <t>Aline, Natália, Ana, thamara (extra)</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>thamara</t>
+  </si>
+  <si>
+    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
+  </si>
+  <si>
+    <t>adnan jamil el homoui</t>
+  </si>
+  <si>
+    <t>Dr. Arthur</t>
+  </si>
+  <si>
+    <t>hipertenso em uso de alodipina</t>
   </si>
   <si>
     <t>Sim</t>
   </si>
   <si>
-    <t>Não</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nega </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fios de 2 e 3 comprimentos médios e grossos </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aline </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natália </t>
-  </si>
-  <si>
-    <t>Xilo sem vaso</t>
-  </si>
-  <si>
-    <t>A dra aqui faz um bloqueio diferente uma seringa de 3 ml 1,5 de xilo e 1,5 de soro 
-E duas seringas  de 1,5 ropi e 1,5 de soro</t>
-  </si>
-  <si>
-    <t>{"tipo":"Xilo sem vaso","seringas":"3","comentarios":"A dra aqui faz um bloqueio diferente uma seringa de 3 ml 1,5 de xilo e 1,5 de soro \nE duas seringas  de 1,5 ropi e 1,5 de soro"}</t>
-  </si>
-  <si>
-    <t>2025-03-06</t>
-  </si>
-  <si>
-    <t>05/03/2025</t>
-  </si>
-  <si>
-    <t>Jonas Galatti Carbonera</t>
-  </si>
-  <si>
-    <t>Ribeirão Preto</t>
-  </si>
-  <si>
-    <t>Dr. Daniel</t>
-  </si>
-  <si>
-    <t>Aline, Natália, Ana, thamara (extra)</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>thamara</t>
-  </si>
-  <si>
-    <t>{"tipo":"Não","seringas":"","comentarios":""}</t>
-  </si>
-  <si>
-    <t>adnan jamil el homoui</t>
-  </si>
-  <si>
-    <t>Dr. Arthur</t>
-  </si>
-  <si>
-    <t>hipertenso em uso de alodipina</t>
+    <t>has</t>
   </si>
   <si>
     <t>Hygor Henrique Bonfante</t>
@@ -316,6 +276,12 @@
 </t>
   </si>
   <si>
+    <t>2025-03-10</t>
+  </si>
+  <si>
+    <t>09/03/2025</t>
+  </si>
+  <si>
     <t>Weslei Diego Pavini</t>
   </si>
   <si>
@@ -349,67 +315,108 @@
     <t>José Antônio Tonetto Neto</t>
   </si>
   <si>
-    <t>6.5</t>
-  </si>
-  <si>
-    <t>3498</t>
-  </si>
-  <si>
-    <t>808</t>
-  </si>
-  <si>
-    <t>33</t>
+    <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Douglas Rodrigues Costa </t>
+  </si>
+  <si>
+    <t>2025-03-12</t>
+  </si>
+  <si>
+    <t>11/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedro Rafael de Almeida Picaccio </t>
+  </si>
+  <si>
+    <t>io 1 e 2 Fios finos e curtos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rodolfo Carola </t>
+  </si>
+  <si>
+    <t>fio 1 e 2 Fios de espessura média e comprimento médio</t>
+  </si>
+  <si>
+    <t>Alan Ribeiro de Paula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 1 e 2 Fios de espessura grossa e comprimento longo.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucas Colleoni Ruaro </t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>3800</t>
+  </si>
+  <si>
+    <t>2505</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>1105</t>
+  </si>
+  <si>
+    <t>190</t>
+  </si>
+  <si>
+    <t>0.85</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>1750</t>
   </si>
   <si>
     <t>1500</t>
   </si>
   <si>
-    <t>1190</t>
-  </si>
-  <si>
-    <t>0.95</t>
+    <t>114</t>
+  </si>
+  <si>
+    <t>1450</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>450</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>700</t>
-  </si>
-  <si>
-    <t>668</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>1050</t>
-  </si>
-  <si>
-    <t>930</t>
-  </si>
-  <si>
-    <t>1300</t>
-  </si>
-  <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>57</t>
-  </si>
-  <si>
-    <t>750</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fio 1 e 2 Fios fino e longo.
+    <t>3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 1 e 2 Fios de espessura fina e comprimento curto.
 </t>
   </si>
 </sst>
@@ -773,12 +780,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH9"/>
+  <dimension ref="A1:BH14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
@@ -986,28 +991,13 @@
         <v>66</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>3414</v>
+        <v>3705</v>
       </c>
       <c r="J2">
-        <v>2964</v>
-      </c>
-      <c r="K2">
-        <v>80</v>
-      </c>
-      <c r="L2">
-        <v>450</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>200</v>
-      </c>
-      <c r="O2">
-        <v>200</v>
+        <v>3705</v>
       </c>
       <c r="P2" t="s">
         <v>67</v>
@@ -1016,49 +1006,46 @@
         <v>0.85</v>
       </c>
       <c r="R2">
-        <v>6</v>
-      </c>
-      <c r="S2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="V2">
-        <v>650</v>
+        <v>750</v>
       </c>
       <c r="W2">
-        <v>637</v>
+        <v>730</v>
       </c>
       <c r="X2">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="Y2">
-        <v>1150</v>
+        <v>1250</v>
       </c>
       <c r="Z2">
-        <v>1027</v>
+        <v>1202</v>
       </c>
       <c r="AA2">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="AB2">
         <v>1200</v>
       </c>
       <c r="AC2">
-        <v>1100</v>
+        <v>1186</v>
       </c>
       <c r="AD2">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AE2">
-        <v>700</v>
+        <v>630</v>
       </c>
       <c r="AF2">
-        <v>650</v>
+        <v>587</v>
       </c>
       <c r="AG2">
         <v>1</v>
@@ -1070,123 +1057,114 @@
         <v>1</v>
       </c>
       <c r="AJ2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ2" t="s">
         <v>68</v>
       </c>
-      <c r="AK2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO2" t="s">
+      <c r="AS2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH2" t="s">
         <v>69</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>73</v>
-      </c>
-      <c r="AT2">
-        <v>3</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>74</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G3" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H3">
         <v>5</v>
       </c>
       <c r="I3">
-        <v>3705</v>
+        <v>2850</v>
       </c>
       <c r="J3">
-        <v>3705</v>
+        <v>100</v>
+      </c>
+      <c r="N3">
+        <v>310</v>
+      </c>
+      <c r="O3">
+        <v>240</v>
       </c>
       <c r="P3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q3">
         <v>0.85</v>
       </c>
       <c r="R3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="T3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U3">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="V3">
-        <v>750</v>
+        <v>630</v>
       </c>
       <c r="W3">
-        <v>730</v>
+        <v>585</v>
       </c>
       <c r="X3">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="Y3">
-        <v>1250</v>
+        <v>1120</v>
       </c>
       <c r="Z3">
-        <v>1202</v>
+        <v>1090</v>
       </c>
       <c r="AA3">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="AB3">
         <v>1200</v>
       </c>
       <c r="AC3">
-        <v>1186</v>
+        <v>1060</v>
       </c>
       <c r="AD3">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="AE3">
-        <v>630</v>
+        <v>750</v>
       </c>
       <c r="AF3">
-        <v>587</v>
+        <v>885</v>
       </c>
       <c r="AG3">
         <v>1</v>
@@ -1195,72 +1173,78 @@
         <v>1</v>
       </c>
       <c r="AI3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AJ3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AQ3" t="s">
         <v>68</v>
       </c>
-      <c r="AK3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>83</v>
-      </c>
       <c r="AS3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH3" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H4">
         <v>5</v>
       </c>
       <c r="I4">
+        <v>3400</v>
+      </c>
+      <c r="J4">
         <v>2850</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>100</v>
       </c>
       <c r="N4">
         <v>310</v>
       </c>
       <c r="O4">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q4">
         <v>0.85</v>
@@ -1269,7 +1253,7 @@
         <v>3</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="U4">
         <v>45</v>
@@ -1305,7 +1289,7 @@
         <v>750</v>
       </c>
       <c r="AF4">
-        <v>885</v>
+        <v>665</v>
       </c>
       <c r="AG4">
         <v>1</v>
@@ -1317,54 +1301,54 @@
         <v>3</v>
       </c>
       <c r="AJ4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>74</v>
+      </c>
+      <c r="AQ4" t="s">
         <v>68</v>
       </c>
-      <c r="AK4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>83</v>
-      </c>
       <c r="AS4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH4" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -1385,7 +1369,7 @@
         <v>2</v>
       </c>
       <c r="P5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q5">
         <v>0.85</v>
@@ -1442,57 +1426,57 @@
         <v>2</v>
       </c>
       <c r="AJ5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ5" t="s">
         <v>68</v>
       </c>
-      <c r="AK5" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>89</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>90</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>83</v>
-      </c>
       <c r="AS5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH5" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="F6" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="G6" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -1513,7 +1497,7 @@
         <v>200</v>
       </c>
       <c r="P6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q6">
         <v>0.85</v>
@@ -1573,57 +1557,57 @@
         <v>1</v>
       </c>
       <c r="AJ6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>83</v>
+      </c>
+      <c r="AQ6" t="s">
         <v>68</v>
       </c>
-      <c r="AK6" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL6" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM6" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN6" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>89</v>
-      </c>
-      <c r="AP6" t="s">
-        <v>96</v>
-      </c>
-      <c r="AQ6" t="s">
-        <v>83</v>
-      </c>
       <c r="AS6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH6" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="G7" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H7">
         <v>5</v>
@@ -1647,7 +1631,7 @@
         <v>98</v>
       </c>
       <c r="P7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q7">
         <v>0.85</v>
@@ -1707,54 +1691,54 @@
         <v>2</v>
       </c>
       <c r="AJ7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AK7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AL7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AM7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AN7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AQ7" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="AR7" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="AS7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH7" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="F8" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="G8" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H8">
         <v>6.5</v>
@@ -1769,7 +1753,7 @@
         <v>80</v>
       </c>
       <c r="P8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q8">
         <v>0.85</v>
@@ -1826,168 +1810,826 @@
         <v>2</v>
       </c>
       <c r="AJ8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AK8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AL8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AM8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AN8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AP8" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="AQ8" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="AR8" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="AS8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="BH8" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9">
+        <v>6.5</v>
+      </c>
+      <c r="I9">
+        <v>3498</v>
+      </c>
+      <c r="J9">
+        <v>808</v>
+      </c>
+      <c r="K9">
+        <v>33</v>
+      </c>
+      <c r="L9">
+        <v>1500</v>
+      </c>
+      <c r="M9">
+        <v>1190</v>
+      </c>
+      <c r="P9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q9">
+        <v>0.95</v>
+      </c>
+      <c r="R9">
+        <v>2</v>
+      </c>
+      <c r="S9">
+        <v>7</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9">
+        <v>64</v>
+      </c>
+      <c r="V9">
+        <v>700</v>
+      </c>
+      <c r="W9">
+        <v>668</v>
+      </c>
+      <c r="X9">
+        <v>76</v>
+      </c>
+      <c r="Y9">
+        <v>1050</v>
+      </c>
+      <c r="Z9">
+        <v>930</v>
+      </c>
+      <c r="AA9">
+        <v>76</v>
+      </c>
+      <c r="AB9">
+        <v>1300</v>
+      </c>
+      <c r="AC9">
+        <v>1200</v>
+      </c>
+      <c r="AD9">
+        <v>57</v>
+      </c>
+      <c r="AE9">
+        <v>750</v>
+      </c>
+      <c r="AF9">
+        <v>700</v>
+      </c>
+      <c r="AG9">
+        <v>1</v>
+      </c>
+      <c r="AH9">
+        <v>2</v>
+      </c>
+      <c r="AI9">
+        <v>2</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10">
+        <v>6.5</v>
+      </c>
+      <c r="I10">
+        <v>4000</v>
+      </c>
+      <c r="J10">
+        <v>2710</v>
+      </c>
+      <c r="K10">
+        <v>99</v>
+      </c>
+      <c r="L10">
+        <v>773</v>
+      </c>
+      <c r="M10">
+        <v>517</v>
+      </c>
+      <c r="P10" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q10">
+        <v>0.95</v>
+      </c>
+      <c r="R10">
+        <v>6</v>
+      </c>
+      <c r="S10">
+        <v>7</v>
+      </c>
+      <c r="T10">
+        <v>1</v>
+      </c>
+      <c r="U10">
+        <v>40</v>
+      </c>
+      <c r="V10">
+        <v>450</v>
+      </c>
+      <c r="W10">
+        <v>360</v>
+      </c>
+      <c r="X10">
+        <v>100</v>
+      </c>
+      <c r="Y10">
+        <v>1700</v>
+      </c>
+      <c r="Z10">
+        <v>1590</v>
+      </c>
+      <c r="AA10">
+        <v>100</v>
+      </c>
+      <c r="AB10">
+        <v>1650</v>
+      </c>
+      <c r="AC10">
+        <v>1544</v>
+      </c>
+      <c r="AD10">
+        <v>41</v>
+      </c>
+      <c r="AE10">
+        <v>600</v>
+      </c>
+      <c r="AF10">
+        <v>503</v>
+      </c>
+      <c r="AG10">
+        <v>2</v>
+      </c>
+      <c r="AH10">
+        <v>2</v>
+      </c>
+      <c r="AI10">
+        <v>3</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>76</v>
+      </c>
+      <c r="AQ10" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11">
+        <v>7</v>
+      </c>
+      <c r="I11">
+        <v>4222</v>
+      </c>
+      <c r="J11">
+        <v>3872</v>
+      </c>
+      <c r="K11">
+        <v>108</v>
+      </c>
+      <c r="N11">
+        <v>180</v>
+      </c>
+      <c r="O11">
+        <v>170</v>
+      </c>
+      <c r="P11" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q11">
+        <v>0.85</v>
+      </c>
+      <c r="R11">
+        <v>8</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="U11">
+        <v>50</v>
+      </c>
+      <c r="V11">
+        <v>700</v>
+      </c>
+      <c r="W11">
+        <v>647</v>
+      </c>
+      <c r="X11">
+        <v>83</v>
+      </c>
+      <c r="Y11">
+        <v>1640</v>
+      </c>
+      <c r="Z11">
+        <v>1575</v>
+      </c>
+      <c r="AA11">
+        <v>83</v>
+      </c>
+      <c r="AB11">
+        <v>1650</v>
+      </c>
+      <c r="AC11">
+        <v>1600</v>
+      </c>
+      <c r="AD11">
+        <v>50</v>
+      </c>
+      <c r="AE11">
+        <v>459</v>
+      </c>
+      <c r="AF11">
+        <v>400</v>
+      </c>
+      <c r="AG11">
+        <v>2</v>
+      </c>
+      <c r="AH11">
+        <v>2</v>
+      </c>
+      <c r="AI11">
+        <v>3</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN11" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>102</v>
+      </c>
+      <c r="AQ11" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS11" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12">
+        <v>6.5</v>
+      </c>
+      <c r="I12">
+        <v>3630</v>
+      </c>
+      <c r="J12">
+        <v>3464</v>
+      </c>
+      <c r="K12">
+        <v>123</v>
+      </c>
+      <c r="N12">
+        <v>85</v>
+      </c>
+      <c r="O12">
+        <v>81</v>
+      </c>
+      <c r="P12" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q12">
+        <v>0.85</v>
+      </c>
+      <c r="R12">
+        <v>5</v>
+      </c>
+      <c r="T12">
+        <v>1</v>
+      </c>
+      <c r="U12">
+        <v>60</v>
+      </c>
+      <c r="V12">
+        <v>500</v>
+      </c>
+      <c r="W12">
+        <v>433</v>
+      </c>
+      <c r="X12">
+        <v>90</v>
+      </c>
+      <c r="Y12">
+        <v>1550</v>
+      </c>
+      <c r="Z12">
+        <v>1450</v>
+      </c>
+      <c r="AA12">
+        <v>93</v>
+      </c>
+      <c r="AB12">
+        <v>1300</v>
+      </c>
+      <c r="AC12">
+        <v>1210</v>
+      </c>
+      <c r="AD12">
+        <v>68</v>
+      </c>
+      <c r="AE12">
+        <v>600</v>
+      </c>
+      <c r="AF12">
+        <v>537</v>
+      </c>
+      <c r="AG12">
+        <v>2</v>
+      </c>
+      <c r="AH12">
+        <v>2</v>
+      </c>
+      <c r="AI12">
+        <v>2</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>73</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP12" t="s">
+        <v>104</v>
+      </c>
+      <c r="AQ12" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR12" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS12" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s">
         <v>105</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>87</v>
+      </c>
+      <c r="G13" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13">
+        <v>6</v>
+      </c>
+      <c r="I13">
+        <v>3710</v>
+      </c>
+      <c r="J13">
+        <v>3100</v>
+      </c>
+      <c r="K13">
+        <v>113</v>
+      </c>
+      <c r="L13">
+        <v>425</v>
+      </c>
+      <c r="M13">
+        <v>185</v>
+      </c>
+      <c r="P13" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q13">
+        <v>0.85</v>
+      </c>
+      <c r="R13">
+        <v>7</v>
+      </c>
+      <c r="S13">
+        <v>6</v>
+      </c>
+      <c r="T13">
+        <v>-3</v>
+      </c>
+      <c r="U13">
+        <v>59</v>
+      </c>
+      <c r="V13">
+        <v>700</v>
+      </c>
+      <c r="W13">
+        <v>662</v>
+      </c>
+      <c r="X13">
+        <v>76</v>
+      </c>
+      <c r="Y13">
+        <v>1420</v>
+      </c>
+      <c r="Z13">
+        <v>1378</v>
+      </c>
+      <c r="AA13">
+        <v>76</v>
+      </c>
+      <c r="AB13">
+        <v>1430</v>
+      </c>
+      <c r="AC13">
+        <v>1200</v>
+      </c>
+      <c r="AD13">
+        <v>52</v>
+      </c>
+      <c r="AE13">
+        <v>500</v>
+      </c>
+      <c r="AF13">
+        <v>470</v>
+      </c>
+      <c r="AG13">
+        <v>2</v>
+      </c>
+      <c r="AH13">
+        <v>1</v>
+      </c>
+      <c r="AI13">
+        <v>3</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP13" t="s">
         <v>106</v>
       </c>
-      <c r="C9" t="s">
+      <c r="AQ13" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" t="s">
         <v>107</v>
       </c>
-      <c r="D9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E9" t="s">
-        <v>80</v>
-      </c>
-      <c r="F9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="D14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s">
         <v>82</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H14" t="s">
         <v>108</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I14" t="s">
         <v>109</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J14" t="s">
         <v>110</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K14" t="s">
         <v>111</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L14" t="s">
         <v>112</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M14" t="s">
         <v>113</v>
       </c>
-      <c r="P9" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q9" t="s">
+      <c r="P14" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q14" t="s">
         <v>114</v>
       </c>
-      <c r="R9" t="s">
+      <c r="R14" t="s">
         <v>115</v>
       </c>
-      <c r="S9" t="s">
+      <c r="S14" t="s">
         <v>116</v>
       </c>
-      <c r="T9" t="s">
+      <c r="T14" t="s">
+        <v>116</v>
+      </c>
+      <c r="U14" t="s">
         <v>117</v>
       </c>
-      <c r="U9" t="s">
+      <c r="V14" t="s">
         <v>118</v>
       </c>
-      <c r="V9" t="s">
+      <c r="W14" t="s">
         <v>119</v>
       </c>
-      <c r="W9" t="s">
+      <c r="X14" t="s">
         <v>120</v>
       </c>
-      <c r="X9" t="s">
+      <c r="Y14" t="s">
         <v>121</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z14" t="s">
         <v>122</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA14" t="s">
         <v>123</v>
       </c>
-      <c r="AA9" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB9" t="s">
+      <c r="AB14" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC14" t="s">
         <v>124</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AD14" t="s">
         <v>125</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AE14" t="s">
         <v>126</v>
       </c>
-      <c r="AE9" t="s">
+      <c r="AF14" t="s">
         <v>127</v>
       </c>
-      <c r="AF9" t="s">
-        <v>119</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>117</v>
-      </c>
-      <c r="AH9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN9" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO9" t="s">
+      <c r="AG14" t="s">
+        <v>128</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>130</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR14" t="s">
         <v>89</v>
       </c>
-      <c r="AP9" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ9" t="s">
-        <v>99</v>
-      </c>
-      <c r="AR9" t="s">
-        <v>100</v>
-      </c>
-      <c r="AS9" t="s">
-        <v>68</v>
-      </c>
-      <c r="BH9" t="s">
-        <v>84</v>
+      <c r="AS14" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH14" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update patient data in surgery report; added 3 new patients.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/relatorio_cirurgias.xlsx
+++ b/attached_assets/relatorio_cirurgias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Usuários\Arthur\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{846924BB-0F6A-4F6A-B5F5-401829AAEA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ADF91A9-9857-40E3-B71D-E19CF7E62309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="119">
   <si>
     <t>data</t>
   </si>
@@ -350,73 +350,39 @@
     <t xml:space="preserve">Lucas Colleoni Ruaro </t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>3800</t>
-  </si>
-  <si>
-    <t>2505</t>
-  </si>
-  <si>
-    <t>106</t>
-  </si>
-  <si>
-    <t>1105</t>
-  </si>
-  <si>
-    <t>190</t>
-  </si>
-  <si>
-    <t>0.85</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>700</t>
-  </si>
-  <si>
-    <t>400</t>
-  </si>
-  <si>
-    <t>117</t>
-  </si>
-  <si>
-    <t>1750</t>
-  </si>
-  <si>
-    <t>1500</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>1450</t>
-  </si>
-  <si>
-    <t>67</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>450</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t xml:space="preserve">fio 1 e 2 Fios de espessura fina e comprimento curto.
+</t>
+  </si>
+  <si>
+    <t>2025-03-14</t>
+  </si>
+  <si>
+    <t>13/03/2025</t>
+  </si>
+  <si>
+    <t>Lucas Evandro de Melo</t>
+  </si>
+  <si>
+    <t>Darcilio Maester Neto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 1 e 2 Fios de espessura grosso e comprimento longo.
+</t>
+  </si>
+  <si>
+    <t>2025-03-17</t>
+  </si>
+  <si>
+    <t>16/03/2025</t>
+  </si>
+  <si>
+    <t>Thiago Domingos Chicarelli</t>
+  </si>
+  <si>
+    <t>Aline, Natália, Ana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fio 1 e 2 Fios de espessura média e comprimento médio.
 </t>
   </si>
 </sst>
@@ -780,11 +746,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH14"/>
+  <dimension ref="A1:BH17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="31.42578125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -2523,83 +2486,83 @@
       <c r="G14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" t="s">
-        <v>108</v>
-      </c>
-      <c r="I14" t="s">
-        <v>109</v>
-      </c>
-      <c r="J14" t="s">
-        <v>110</v>
-      </c>
-      <c r="K14" t="s">
-        <v>111</v>
-      </c>
-      <c r="L14" t="s">
-        <v>112</v>
-      </c>
-      <c r="M14" t="s">
-        <v>113</v>
+      <c r="H14">
+        <v>6</v>
+      </c>
+      <c r="I14">
+        <v>3800</v>
+      </c>
+      <c r="J14">
+        <v>2505</v>
+      </c>
+      <c r="K14">
+        <v>106</v>
+      </c>
+      <c r="L14">
+        <v>1105</v>
+      </c>
+      <c r="M14">
+        <v>190</v>
       </c>
       <c r="P14" t="s">
         <v>67</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="Q14">
+        <v>0.85</v>
+      </c>
+      <c r="R14">
+        <v>7</v>
+      </c>
+      <c r="S14">
+        <v>1</v>
+      </c>
+      <c r="T14">
+        <v>1</v>
+      </c>
+      <c r="U14">
+        <v>70</v>
+      </c>
+      <c r="V14">
+        <v>700</v>
+      </c>
+      <c r="W14">
+        <v>400</v>
+      </c>
+      <c r="X14">
+        <v>117</v>
+      </c>
+      <c r="Y14">
+        <v>1750</v>
+      </c>
+      <c r="Z14">
+        <v>1500</v>
+      </c>
+      <c r="AA14">
         <v>114</v>
       </c>
-      <c r="R14" t="s">
-        <v>115</v>
-      </c>
-      <c r="S14" t="s">
-        <v>116</v>
-      </c>
-      <c r="T14" t="s">
-        <v>116</v>
-      </c>
-      <c r="U14" t="s">
-        <v>117</v>
-      </c>
-      <c r="V14" t="s">
-        <v>118</v>
-      </c>
-      <c r="W14" t="s">
-        <v>119</v>
-      </c>
-      <c r="X14" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>121</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>122</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>123</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC14" t="s">
-        <v>124</v>
-      </c>
-      <c r="AD14" t="s">
-        <v>125</v>
-      </c>
-      <c r="AE14" t="s">
-        <v>126</v>
-      </c>
-      <c r="AF14" t="s">
-        <v>127</v>
-      </c>
-      <c r="AG14" t="s">
-        <v>128</v>
-      </c>
-      <c r="AH14" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI14" t="s">
-        <v>129</v>
+      <c r="AB14">
+        <v>1500</v>
+      </c>
+      <c r="AC14">
+        <v>1450</v>
+      </c>
+      <c r="AD14">
+        <v>67</v>
+      </c>
+      <c r="AE14">
+        <v>500</v>
+      </c>
+      <c r="AF14">
+        <v>450</v>
+      </c>
+      <c r="AG14">
+        <v>2</v>
+      </c>
+      <c r="AH14">
+        <v>2</v>
+      </c>
+      <c r="AI14">
+        <v>3</v>
       </c>
       <c r="AJ14" t="s">
         <v>67</v>
@@ -2617,7 +2580,7 @@
         <v>67</v>
       </c>
       <c r="AO14" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="AQ14" t="s">
         <v>88</v>
@@ -2629,6 +2592,375 @@
         <v>67</v>
       </c>
       <c r="BH14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>82</v>
+      </c>
+      <c r="H15">
+        <v>7</v>
+      </c>
+      <c r="I15">
+        <v>4070</v>
+      </c>
+      <c r="J15">
+        <v>4070</v>
+      </c>
+      <c r="K15">
+        <v>88</v>
+      </c>
+      <c r="P15" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q15">
+        <v>0.85</v>
+      </c>
+      <c r="R15">
+        <v>6</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15">
+        <v>45</v>
+      </c>
+      <c r="V15">
+        <v>600</v>
+      </c>
+      <c r="W15">
+        <v>550</v>
+      </c>
+      <c r="X15">
+        <v>96</v>
+      </c>
+      <c r="Y15">
+        <v>1600</v>
+      </c>
+      <c r="Z15">
+        <v>1550</v>
+      </c>
+      <c r="AA15">
+        <v>96</v>
+      </c>
+      <c r="AB15">
+        <v>1700</v>
+      </c>
+      <c r="AC15">
+        <v>1500</v>
+      </c>
+      <c r="AD15">
+        <v>45</v>
+      </c>
+      <c r="AE15">
+        <v>600</v>
+      </c>
+      <c r="AF15">
+        <v>550</v>
+      </c>
+      <c r="AG15">
+        <v>2</v>
+      </c>
+      <c r="AH15">
+        <v>1</v>
+      </c>
+      <c r="AI15">
+        <v>3</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN15" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS15" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" t="s">
+        <v>66</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="I16">
+        <v>3700</v>
+      </c>
+      <c r="J16">
+        <v>3700</v>
+      </c>
+      <c r="K16">
+        <v>127</v>
+      </c>
+      <c r="P16" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q16">
+        <v>0.85</v>
+      </c>
+      <c r="R16">
+        <v>7</v>
+      </c>
+      <c r="T16">
+        <v>1</v>
+      </c>
+      <c r="U16">
+        <v>52</v>
+      </c>
+      <c r="V16">
+        <v>600</v>
+      </c>
+      <c r="W16">
+        <v>563</v>
+      </c>
+      <c r="X16">
+        <v>76</v>
+      </c>
+      <c r="Y16">
+        <v>1300</v>
+      </c>
+      <c r="Z16">
+        <v>1200</v>
+      </c>
+      <c r="AA16">
+        <v>81</v>
+      </c>
+      <c r="AB16">
+        <v>1500</v>
+      </c>
+      <c r="AC16">
+        <v>1400</v>
+      </c>
+      <c r="AD16">
+        <v>42</v>
+      </c>
+      <c r="AE16">
+        <v>550</v>
+      </c>
+      <c r="AF16">
+        <v>537</v>
+      </c>
+      <c r="AG16">
+        <v>2</v>
+      </c>
+      <c r="AH16">
+        <v>2</v>
+      </c>
+      <c r="AI16">
+        <v>3</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>73</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN16" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>113</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR16" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS16" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:60" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" t="s">
+        <v>117</v>
+      </c>
+      <c r="G17" t="s">
+        <v>66</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>2513</v>
+      </c>
+      <c r="J17">
+        <v>2253</v>
+      </c>
+      <c r="K17">
+        <v>52</v>
+      </c>
+      <c r="N17">
+        <v>130</v>
+      </c>
+      <c r="O17">
+        <v>130</v>
+      </c>
+      <c r="P17" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q17">
+        <v>0.85</v>
+      </c>
+      <c r="R17">
+        <v>4</v>
+      </c>
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>58</v>
+      </c>
+      <c r="V17">
+        <v>470</v>
+      </c>
+      <c r="W17">
+        <v>435</v>
+      </c>
+      <c r="X17">
+        <v>71</v>
+      </c>
+      <c r="Y17">
+        <v>1070</v>
+      </c>
+      <c r="Z17">
+        <v>1022</v>
+      </c>
+      <c r="AA17">
+        <v>68</v>
+      </c>
+      <c r="AB17">
+        <v>580</v>
+      </c>
+      <c r="AC17">
+        <v>482</v>
+      </c>
+      <c r="AD17">
+        <v>52</v>
+      </c>
+      <c r="AE17">
+        <v>660</v>
+      </c>
+      <c r="AF17">
+        <v>580</v>
+      </c>
+      <c r="AG17">
+        <v>1</v>
+      </c>
+      <c r="AH17">
+        <v>1</v>
+      </c>
+      <c r="AI17">
+        <v>1</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN17" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>118</v>
+      </c>
+      <c r="AS17" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH17" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>